<commit_message>
Setup targets, data and model functions prepped and ran
</commit_message>
<xml_diff>
--- a/data/study_characteristics.xlsx
+++ b/data/study_characteristics.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Dropbox\Research\PhD Students\Current\Bailey\exercise_recovery_modalities_meta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A31095-8D1B-4D51-B931-981BE31E4DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{651F1B66-8ECF-4A47-83AE-A87B0AC69A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{9BCA5C17-8C5F-0F4E-86BF-A7E8EC5FB0C0}"/>
+    <workbookView xWindow="4950" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{9BCA5C17-8C5F-0F4E-86BF-A7E8EC5FB0C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$E$1:$E$121</definedName>
+  </definedNames>
   <calcPr calcId="191028" calcMode="manual"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="235">
   <si>
     <t>study id</t>
   </si>
@@ -50,9 +53,6 @@
     <t xml:space="preserve">author </t>
   </si>
   <si>
-    <t xml:space="preserve">mode </t>
-  </si>
-  <si>
     <t>protocol</t>
   </si>
   <si>
@@ -65,60 +65,33 @@
     <t xml:space="preserve">Brown et al. </t>
   </si>
   <si>
-    <t>Compression - custom</t>
-  </si>
-  <si>
     <t>worn immediately after exercise until 48hours</t>
   </si>
   <si>
-    <t>Compression - standard</t>
-  </si>
-  <si>
-    <t>PLA</t>
-  </si>
-  <si>
     <t xml:space="preserve">ultrasound treatment as placebo </t>
   </si>
   <si>
-    <t>SHAM</t>
-  </si>
-  <si>
     <t>The effect of individualised post-exercise blood flow restriction on recovery following strenuous resistance exercise: A randomised controlled trial.</t>
   </si>
   <si>
     <t xml:space="preserve">Leszczynski et al. </t>
   </si>
   <si>
-    <t xml:space="preserve">BFR </t>
-  </si>
-  <si>
     <t>80% AOP 3x5min bouts</t>
   </si>
   <si>
     <t>20mmHg 3x5min bouts</t>
   </si>
   <si>
-    <t>Cold water immersion</t>
-  </si>
-  <si>
-    <t>CON</t>
-  </si>
-  <si>
     <t>15 min passive rest</t>
   </si>
   <si>
-    <t xml:space="preserve">CWI </t>
-  </si>
-  <si>
     <t>Lower-body compression garments worn following exercise improves perceived recovery but not subsequent performance in basketball athletes</t>
   </si>
   <si>
     <t>Atkins et al.</t>
   </si>
   <si>
-    <t>Compression</t>
-  </si>
-  <si>
     <t>worn for 15 hours after exercise</t>
   </si>
   <si>
@@ -131,9 +104,6 @@
     <t>Tanaka et al.</t>
   </si>
   <si>
-    <t>rBFR</t>
-  </si>
-  <si>
     <t xml:space="preserve">BFR at 100% systolic bp applied during 90 sec rest intervals </t>
   </si>
   <si>
@@ -158,9 +128,6 @@
     <t xml:space="preserve">CK only outcome variable - previously determined </t>
   </si>
   <si>
-    <t>Warm water immersion</t>
-  </si>
-  <si>
     <t>30 mins at 38 degrees</t>
   </si>
   <si>
@@ -179,9 +146,6 @@
     <t>0.5 hrs represents post intervention, 0hrs = post exercise</t>
   </si>
   <si>
-    <t xml:space="preserve">Cold therapy </t>
-  </si>
-  <si>
     <t>20 minutes with ice packs and cold towels applied</t>
   </si>
   <si>
@@ -194,27 +158,15 @@
     <t>Arriel et al.</t>
   </si>
   <si>
-    <t>BFR 2x5min</t>
-  </si>
-  <si>
     <t>50mmHG above systolic pressure 2x5 min</t>
   </si>
   <si>
-    <t>SHAM 2x5min</t>
-  </si>
-  <si>
     <t>20mmHg 2x5min bouts</t>
   </si>
   <si>
-    <t>BFR 5x2min</t>
-  </si>
-  <si>
     <t>50mmHG above systolic pressure 5x2 min</t>
   </si>
   <si>
-    <t>SHAM 5x2 min</t>
-  </si>
-  <si>
     <t>20mmHg 5x2min bouts</t>
   </si>
   <si>
@@ -254,9 +206,6 @@
     <t>French et al.</t>
   </si>
   <si>
-    <t>Contrast Therapy</t>
-  </si>
-  <si>
     <t>4x (8-10 degrees for 60secs )then 3x( 37-40 for 180secs)</t>
   </si>
   <si>
@@ -269,24 +218,15 @@
     <t>No recovery intervention</t>
   </si>
   <si>
-    <t>Active</t>
-  </si>
-  <si>
     <t>Effects of air-pulsed cryotherapy on neuromuscular recovery subsequent to exercise-induced muscle damage.</t>
   </si>
   <si>
     <t>Guilhem et al.</t>
   </si>
   <si>
-    <t>Cryotherapy</t>
-  </si>
-  <si>
     <t>3x4 min at -30 degrees</t>
   </si>
   <si>
-    <t>Control</t>
-  </si>
-  <si>
     <t>Passive rest</t>
   </si>
   <si>
@@ -329,9 +269,6 @@
     <t>de Paiva et al.</t>
   </si>
   <si>
-    <t>Cryotherapy (cold therapy)</t>
-  </si>
-  <si>
     <t>Ice packs applied for 20 min</t>
   </si>
   <si>
@@ -413,27 +350,15 @@
     <t>Petrofsky et al.</t>
   </si>
   <si>
-    <t>Cold immediate</t>
-  </si>
-  <si>
     <t>Cold wrap for 20 mins</t>
   </si>
   <si>
-    <t>Cold delayed</t>
-  </si>
-  <si>
     <t>Cold wrap for 20 mins 24 hours post exercise</t>
   </si>
   <si>
-    <t>Heat Immediate</t>
-  </si>
-  <si>
     <t>Heat wrap for 20 mins</t>
   </si>
   <si>
-    <t>Heat Delayed</t>
-  </si>
-  <si>
     <t>Heat wrap for 20 mins 24 hours post exercise</t>
   </si>
   <si>
@@ -452,9 +377,6 @@
     <t>compression conditions excluded as used during exercise</t>
   </si>
   <si>
-    <t>passive</t>
-  </si>
-  <si>
     <t>30 mins passive rest</t>
   </si>
   <si>
@@ -473,9 +395,6 @@
     <t>Anderson et al.</t>
   </si>
   <si>
-    <t>Ice water immersion</t>
-  </si>
-  <si>
     <t>12 min at 5 degrees</t>
   </si>
   <si>
@@ -521,9 +440,6 @@
     <t>30 secs at -60 then 150 secs at -120 1 hour post</t>
   </si>
   <si>
-    <t>Cryotherapy delayed</t>
-  </si>
-  <si>
     <t>31 secs at -60 then 150 secs at -120 4 hours post</t>
   </si>
   <si>
@@ -542,9 +458,6 @@
     <t xml:space="preserve">perception variable excluded - no baseline measure </t>
   </si>
   <si>
-    <t>Massage</t>
-  </si>
-  <si>
     <t>percussive therapy gun</t>
   </si>
   <si>
@@ -605,21 +518,12 @@
     <t>West et al.</t>
   </si>
   <si>
-    <t>G-Trainer</t>
-  </si>
-  <si>
     <t>40% VO2 peak and 75% body weight for 30 mins</t>
   </si>
   <si>
-    <t>Cycling</t>
-  </si>
-  <si>
     <t>40% VO2peak cycling for 30 minutes</t>
   </si>
   <si>
-    <t>Stretching</t>
-  </si>
-  <si>
     <t>30 min stretching protocol</t>
   </si>
   <si>
@@ -698,9 +602,6 @@
     <t>light bench press sessions 6 and 30 hours post</t>
   </si>
   <si>
-    <t xml:space="preserve">Passive </t>
-  </si>
-  <si>
     <t>Effect of CO2 and H2 gas mixture in cold water immersion on recovery after eccentric loading</t>
   </si>
   <si>
@@ -746,9 +647,6 @@
     <t>Wong et al.</t>
   </si>
   <si>
-    <t>BFR</t>
-  </si>
-  <si>
     <t>30,15,15,15 no load at 80% AOP</t>
   </si>
   <si>
@@ -816,6 +714,36 @@
   </si>
   <si>
     <t xml:space="preserve">performance </t>
+  </si>
+  <si>
+    <t>compression</t>
+  </si>
+  <si>
+    <t>placebo</t>
+  </si>
+  <si>
+    <t>cold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contrast </t>
+  </si>
+  <si>
+    <t>bfr</t>
+  </si>
+  <si>
+    <t>control</t>
+  </si>
+  <si>
+    <t>heat</t>
+  </si>
+  <si>
+    <t>contrast</t>
+  </si>
+  <si>
+    <t>massage</t>
+  </si>
+  <si>
+    <t>recovery_mode</t>
   </si>
 </sst>
 </file>
@@ -1203,6 +1131,7 @@
   <dimension ref="A1:H121"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="21.875" customWidth="1"/>
     <col min="3" max="3" width="62.5" customWidth="1"/>
     <col min="4" max="4" width="21.875" customWidth="1"/>
     <col min="5" max="5" width="19.625" customWidth="1"/>
@@ -1226,16 +1155,16 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>234</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
       <c r="H1" t="s">
-        <v>254</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1246,19 +1175,19 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
       <c r="H2" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1269,19 +1198,19 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>225</v>
+      </c>
+      <c r="F3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>10</v>
-      </c>
       <c r="H3" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1292,19 +1221,19 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>226</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H4" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1315,22 +1244,22 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>248</v>
+        <v>213</v>
       </c>
       <c r="D5" t="s">
-        <v>249</v>
+        <v>214</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F5" t="s">
-        <v>105</v>
+        <v>83</v>
       </c>
       <c r="G5" t="s">
-        <v>250</v>
+        <v>215</v>
       </c>
       <c r="H5" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1341,19 +1270,19 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>248</v>
+        <v>213</v>
       </c>
       <c r="D6" t="s">
-        <v>249</v>
+        <v>214</v>
       </c>
       <c r="E6" t="s">
-        <v>72</v>
+        <v>228</v>
       </c>
       <c r="F6" t="s">
-        <v>251</v>
+        <v>216</v>
       </c>
       <c r="H6" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1364,19 +1293,19 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>248</v>
+        <v>213</v>
       </c>
       <c r="D7" t="s">
-        <v>249</v>
+        <v>214</v>
       </c>
       <c r="E7" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="F7" t="s">
-        <v>252</v>
+        <v>217</v>
       </c>
       <c r="H7" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1387,19 +1316,19 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D8" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>229</v>
       </c>
       <c r="F8" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="H8" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1410,19 +1339,19 @@
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>12</v>
+        <v>226</v>
       </c>
       <c r="F9" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="H9" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1433,22 +1362,22 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>243</v>
+        <v>208</v>
       </c>
       <c r="D10" t="s">
-        <v>244</v>
+        <v>209</v>
       </c>
       <c r="E10" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="F10" t="s">
-        <v>245</v>
+        <v>210</v>
       </c>
       <c r="G10" t="s">
-        <v>246</v>
+        <v>211</v>
       </c>
       <c r="H10" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1459,19 +1388,19 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>243</v>
+        <v>208</v>
       </c>
       <c r="D11" t="s">
-        <v>244</v>
+        <v>209</v>
       </c>
       <c r="E11" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F11" t="s">
-        <v>247</v>
+        <v>212</v>
       </c>
       <c r="H11" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1482,19 +1411,19 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>225</v>
       </c>
       <c r="F12" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="H12" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1505,19 +1434,19 @@
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D13" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E13" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F13" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="H13" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1528,22 +1457,22 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E14" t="s">
-        <v>31</v>
+        <v>229</v>
       </c>
       <c r="F14" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="H14" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1554,22 +1483,22 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E15" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F15" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="G15" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="H15" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1580,22 +1509,22 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D16" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="E16" t="s">
-        <v>20</v>
+        <v>227</v>
       </c>
       <c r="F16" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="G16" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="H16" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1606,19 +1535,19 @@
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="E17" t="s">
-        <v>40</v>
+        <v>231</v>
       </c>
       <c r="F17" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="H17" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1629,19 +1558,19 @@
         <v>3</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="E18" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F18" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="H18" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1652,22 +1581,22 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D19" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="E19" t="s">
-        <v>20</v>
+        <v>227</v>
       </c>
       <c r="F19" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="G19" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="H19" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1678,19 +1607,19 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D20" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="E20" t="s">
-        <v>47</v>
+        <v>227</v>
       </c>
       <c r="F20" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="H20" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1701,19 +1630,19 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D21" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="E21" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F21" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="H21" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1724,19 +1653,19 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D22" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="E22" t="s">
-        <v>52</v>
+        <v>229</v>
       </c>
       <c r="F22" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="H22" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -1747,19 +1676,19 @@
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D23" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="E23" t="s">
-        <v>54</v>
+        <v>226</v>
       </c>
       <c r="F23" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="H23" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1770,19 +1699,19 @@
         <v>3</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D24" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="E24" t="s">
-        <v>56</v>
+        <v>229</v>
       </c>
       <c r="F24" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="H24" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1793,19 +1722,19 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D25" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="E25" t="s">
-        <v>58</v>
+        <v>226</v>
       </c>
       <c r="F25" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="H25" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1816,22 +1745,22 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="D26" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="E26" t="s">
-        <v>20</v>
+        <v>227</v>
       </c>
       <c r="F26" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="G26" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="H26" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1842,19 +1771,19 @@
         <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="D27" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="E27" t="s">
-        <v>20</v>
+        <v>227</v>
       </c>
       <c r="F27" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="H27" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -1865,19 +1794,19 @@
         <v>3</v>
       </c>
       <c r="C28" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="D28" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="E28" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F28" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H28" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -1888,22 +1817,22 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="D29" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="E29" t="s">
-        <v>17</v>
+        <v>229</v>
       </c>
       <c r="F29" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="G29" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="H29" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -1914,19 +1843,19 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="D30" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="E30" t="s">
-        <v>14</v>
+        <v>226</v>
       </c>
       <c r="F30" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="H30" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -1937,22 +1866,22 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="D31" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="E31" t="s">
-        <v>72</v>
+        <v>232</v>
       </c>
       <c r="F31" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="G31" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="H31" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1963,19 +1892,19 @@
         <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="D32" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="E32" t="s">
-        <v>26</v>
+        <v>225</v>
       </c>
       <c r="F32" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="H32" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
@@ -1986,19 +1915,19 @@
         <v>3</v>
       </c>
       <c r="C33" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="D33" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="E33" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F33" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H33" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -2009,19 +1938,19 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>239</v>
+        <v>204</v>
       </c>
       <c r="D34" t="s">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="E34" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="F34" t="s">
-        <v>241</v>
+        <v>206</v>
       </c>
       <c r="H34" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -2032,19 +1961,19 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>239</v>
+        <v>204</v>
       </c>
       <c r="D35" t="s">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="E35" t="s">
-        <v>12</v>
+        <v>226</v>
       </c>
       <c r="F35" t="s">
-        <v>242</v>
+        <v>207</v>
       </c>
       <c r="H35" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -2055,19 +1984,19 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="D36" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="E36" t="s">
-        <v>80</v>
+        <v>227</v>
       </c>
       <c r="F36" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="H36" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -2078,19 +2007,19 @@
         <v>2</v>
       </c>
       <c r="C37" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="D37" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="E37" t="s">
-        <v>82</v>
+        <v>230</v>
       </c>
       <c r="F37" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="H37" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -2101,19 +2030,19 @@
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="D38" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="E38" t="s">
-        <v>26</v>
+        <v>225</v>
       </c>
       <c r="F38" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="H38" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -2124,19 +2053,19 @@
         <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="D39" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="E39" t="s">
-        <v>82</v>
+        <v>230</v>
       </c>
       <c r="F39" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="H39" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -2147,19 +2076,19 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>253</v>
+        <v>218</v>
       </c>
       <c r="D40" t="s">
-        <v>235</v>
+        <v>201</v>
       </c>
       <c r="E40" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="F40" t="s">
-        <v>237</v>
+        <v>202</v>
       </c>
       <c r="H40" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -2170,19 +2099,19 @@
         <v>2</v>
       </c>
       <c r="C41" t="s">
-        <v>253</v>
+        <v>218</v>
       </c>
       <c r="D41" t="s">
-        <v>235</v>
+        <v>201</v>
       </c>
       <c r="E41" t="s">
-        <v>14</v>
+        <v>226</v>
       </c>
       <c r="F41" t="s">
-        <v>238</v>
+        <v>203</v>
       </c>
       <c r="H41" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -2193,19 +2122,19 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="D42" t="s">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="E42" t="s">
-        <v>47</v>
+        <v>227</v>
       </c>
       <c r="F42" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="H42" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -2216,19 +2145,19 @@
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="D43" t="s">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="E43" t="s">
-        <v>14</v>
+        <v>226</v>
       </c>
       <c r="F43" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="H43" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -2239,22 +2168,22 @@
         <v>1</v>
       </c>
       <c r="C44" t="s">
-        <v>232</v>
+        <v>198</v>
       </c>
       <c r="D44" t="s">
-        <v>233</v>
+        <v>199</v>
       </c>
       <c r="E44" t="s">
-        <v>26</v>
+        <v>225</v>
       </c>
       <c r="F44" t="s">
-        <v>234</v>
+        <v>200</v>
       </c>
       <c r="G44" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
       <c r="H44" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2265,19 +2194,19 @@
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>232</v>
+        <v>198</v>
       </c>
       <c r="D45" t="s">
-        <v>233</v>
+        <v>199</v>
       </c>
       <c r="E45" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F45" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H45" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -2288,19 +2217,19 @@
         <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>228</v>
+        <v>194</v>
       </c>
       <c r="D46" t="s">
-        <v>229</v>
+        <v>195</v>
       </c>
       <c r="E46" t="s">
-        <v>168</v>
+        <v>233</v>
       </c>
       <c r="F46" t="s">
-        <v>230</v>
+        <v>196</v>
       </c>
       <c r="H46" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -2311,19 +2240,19 @@
         <v>2</v>
       </c>
       <c r="C47" t="s">
-        <v>228</v>
+        <v>194</v>
       </c>
       <c r="D47" t="s">
-        <v>229</v>
+        <v>195</v>
       </c>
       <c r="E47" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="F47" t="s">
-        <v>231</v>
+        <v>197</v>
       </c>
       <c r="H47" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2334,19 +2263,19 @@
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="D48" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="E48" t="s">
-        <v>80</v>
+        <v>227</v>
       </c>
       <c r="F48" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="H48" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -2357,19 +2286,19 @@
         <v>2</v>
       </c>
       <c r="C49" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="D49" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="E49" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F49" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H49" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -2380,22 +2309,22 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="D50" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="E50" t="s">
-        <v>97</v>
+        <v>227</v>
       </c>
       <c r="F50" t="s">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="G50" t="s">
-        <v>99</v>
+        <v>77</v>
       </c>
       <c r="H50" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -2406,19 +2335,19 @@
         <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="D51" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="E51" t="s">
-        <v>12</v>
+        <v>226</v>
       </c>
       <c r="F51" t="s">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="H51" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -2429,19 +2358,19 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="D52" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="E52" t="s">
-        <v>72</v>
+        <v>232</v>
       </c>
       <c r="F52" t="s">
-        <v>103</v>
+        <v>81</v>
       </c>
       <c r="H52" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
@@ -2452,19 +2381,19 @@
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="D53" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="E53" t="s">
-        <v>20</v>
+        <v>227</v>
       </c>
       <c r="F53" t="s">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="H53" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
@@ -2475,19 +2404,19 @@
         <v>3</v>
       </c>
       <c r="C54" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="D54" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="E54" t="s">
-        <v>20</v>
+        <v>227</v>
       </c>
       <c r="F54" t="s">
-        <v>105</v>
+        <v>83</v>
       </c>
       <c r="H54" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -2498,19 +2427,19 @@
         <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="D55" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="E55" t="s">
-        <v>20</v>
+        <v>227</v>
       </c>
       <c r="F55" t="s">
-        <v>106</v>
+        <v>84</v>
       </c>
       <c r="H55" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -2521,19 +2450,19 @@
         <v>5</v>
       </c>
       <c r="C56" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="D56" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="E56" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F56" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="H56" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -2544,19 +2473,19 @@
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="D57" t="s">
+        <v>87</v>
+      </c>
+      <c r="E57" t="s">
         <v>109</v>
       </c>
-      <c r="E57" t="s">
-        <v>77</v>
-      </c>
       <c r="F57" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="H57" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
@@ -2567,19 +2496,19 @@
         <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="D58" t="s">
+        <v>87</v>
+      </c>
+      <c r="E58" t="s">
         <v>109</v>
       </c>
-      <c r="E58" t="s">
-        <v>77</v>
-      </c>
       <c r="F58" t="s">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="H58" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
@@ -2590,19 +2519,19 @@
         <v>3</v>
       </c>
       <c r="C59" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="D59" t="s">
-        <v>109</v>
+        <v>87</v>
       </c>
       <c r="E59" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F59" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H59" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
@@ -2613,22 +2542,22 @@
         <v>1</v>
       </c>
       <c r="C60" t="s">
-        <v>112</v>
+        <v>90</v>
       </c>
       <c r="D60" t="s">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="E60" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F60" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="G60" t="s">
-        <v>115</v>
+        <v>93</v>
       </c>
       <c r="H60" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
@@ -2639,19 +2568,19 @@
         <v>2</v>
       </c>
       <c r="C61" t="s">
-        <v>112</v>
+        <v>90</v>
       </c>
       <c r="D61" t="s">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="E61" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F61" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="H61" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -2662,22 +2591,22 @@
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="D62" t="s">
-        <v>117</v>
+        <v>95</v>
       </c>
       <c r="E62" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F62" t="s">
-        <v>118</v>
+        <v>96</v>
       </c>
       <c r="G62" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="H62" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
@@ -2688,19 +2617,19 @@
         <v>2</v>
       </c>
       <c r="C63" t="s">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="D63" t="s">
-        <v>117</v>
+        <v>95</v>
       </c>
       <c r="E63" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F63" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H63" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
@@ -2711,19 +2640,19 @@
         <v>1</v>
       </c>
       <c r="C64" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D64" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="E64" t="s">
-        <v>26</v>
+        <v>225</v>
       </c>
       <c r="F64" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
       <c r="H64" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
@@ -2734,19 +2663,19 @@
         <v>1</v>
       </c>
       <c r="C65" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="D65" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="E65" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F65" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H65" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
@@ -2757,19 +2686,19 @@
         <v>1</v>
       </c>
       <c r="C66" t="s">
-        <v>123</v>
+        <v>101</v>
       </c>
       <c r="D66" t="s">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="E66" t="s">
-        <v>125</v>
+        <v>227</v>
       </c>
       <c r="F66" t="s">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="H66" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
@@ -2780,19 +2709,19 @@
         <v>2</v>
       </c>
       <c r="C67" t="s">
-        <v>123</v>
+        <v>101</v>
       </c>
       <c r="D67" t="s">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="E67" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
       <c r="F67" t="s">
-        <v>128</v>
+        <v>104</v>
       </c>
       <c r="H67" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
@@ -2803,19 +2732,19 @@
         <v>3</v>
       </c>
       <c r="C68" t="s">
-        <v>123</v>
+        <v>101</v>
       </c>
       <c r="D68" t="s">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="E68" t="s">
-        <v>129</v>
+        <v>231</v>
       </c>
       <c r="F68" t="s">
-        <v>130</v>
+        <v>105</v>
       </c>
       <c r="H68" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
@@ -2826,19 +2755,19 @@
         <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>123</v>
+        <v>101</v>
       </c>
       <c r="D69" t="s">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="E69" t="s">
-        <v>131</v>
+        <v>231</v>
       </c>
       <c r="F69" t="s">
-        <v>132</v>
+        <v>106</v>
       </c>
       <c r="H69" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -2849,19 +2778,19 @@
         <v>5</v>
       </c>
       <c r="C70" t="s">
-        <v>123</v>
+        <v>101</v>
       </c>
       <c r="D70" t="s">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="E70" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F70" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H70" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
@@ -2872,22 +2801,22 @@
         <v>1</v>
       </c>
       <c r="C71" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="D71" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="E71" t="s">
-        <v>135</v>
+        <v>109</v>
       </c>
       <c r="F71" t="s">
-        <v>136</v>
+        <v>110</v>
       </c>
       <c r="G71" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="H71" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
@@ -2898,19 +2827,19 @@
         <v>1</v>
       </c>
       <c r="C72" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="D72" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="E72" t="s">
-        <v>138</v>
+        <v>230</v>
       </c>
       <c r="F72" t="s">
-        <v>139</v>
+        <v>112</v>
       </c>
       <c r="H72" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -2921,19 +2850,19 @@
         <v>1</v>
       </c>
       <c r="C73" t="s">
-        <v>140</v>
+        <v>113</v>
       </c>
       <c r="D73" t="s">
-        <v>141</v>
+        <v>114</v>
       </c>
       <c r="E73" t="s">
-        <v>40</v>
+        <v>231</v>
       </c>
       <c r="F73" t="s">
-        <v>142</v>
+        <v>115</v>
       </c>
       <c r="H73" t="s">
-        <v>258</v>
+        <v>223</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
@@ -2944,19 +2873,19 @@
         <v>2</v>
       </c>
       <c r="C74" t="s">
-        <v>140</v>
+        <v>113</v>
       </c>
       <c r="D74" t="s">
-        <v>141</v>
+        <v>114</v>
       </c>
       <c r="E74" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F74" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H74" t="s">
-        <v>258</v>
+        <v>223</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -2967,19 +2896,19 @@
         <v>1</v>
       </c>
       <c r="C75" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="D75" t="s">
-        <v>144</v>
+        <v>117</v>
       </c>
       <c r="E75" t="s">
-        <v>145</v>
+        <v>227</v>
       </c>
       <c r="F75" t="s">
-        <v>146</v>
+        <v>118</v>
       </c>
       <c r="H75" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -2990,19 +2919,19 @@
         <v>1</v>
       </c>
       <c r="C76" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="D76" t="s">
-        <v>144</v>
+        <v>117</v>
       </c>
       <c r="E76" t="s">
-        <v>20</v>
+        <v>227</v>
       </c>
       <c r="F76" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
       <c r="H76" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
@@ -3013,19 +2942,19 @@
         <v>1</v>
       </c>
       <c r="C77" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="D77" t="s">
-        <v>144</v>
+        <v>117</v>
       </c>
       <c r="E77" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F77" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="H77" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -3036,19 +2965,19 @@
         <v>1</v>
       </c>
       <c r="C78" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
       <c r="D78" t="s">
-        <v>149</v>
+        <v>121</v>
       </c>
       <c r="E78" t="s">
-        <v>72</v>
+        <v>232</v>
       </c>
       <c r="F78" t="s">
-        <v>150</v>
+        <v>122</v>
       </c>
       <c r="H78" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
@@ -3059,19 +2988,19 @@
         <v>1</v>
       </c>
       <c r="C79" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
       <c r="D79" t="s">
-        <v>149</v>
+        <v>121</v>
       </c>
       <c r="E79" t="s">
-        <v>20</v>
+        <v>227</v>
       </c>
       <c r="F79" t="s">
-        <v>151</v>
+        <v>123</v>
       </c>
       <c r="H79" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
@@ -3082,19 +3011,19 @@
         <v>3</v>
       </c>
       <c r="C80" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
       <c r="D80" t="s">
-        <v>149</v>
+        <v>121</v>
       </c>
       <c r="E80" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F80" t="s">
-        <v>152</v>
+        <v>124</v>
       </c>
       <c r="H80" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
@@ -3105,19 +3034,19 @@
         <v>1</v>
       </c>
       <c r="C81" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="D81" t="s">
-        <v>154</v>
+        <v>126</v>
       </c>
       <c r="E81" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="F81" t="s">
-        <v>155</v>
+        <v>127</v>
       </c>
       <c r="H81" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
@@ -3128,19 +3057,19 @@
         <v>2</v>
       </c>
       <c r="C82" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="D82" t="s">
-        <v>154</v>
+        <v>126</v>
       </c>
       <c r="E82" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="F82" t="s">
-        <v>156</v>
+        <v>128</v>
       </c>
       <c r="H82" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
@@ -3151,19 +3080,19 @@
         <v>3</v>
       </c>
       <c r="C83" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="D83" t="s">
-        <v>154</v>
+        <v>126</v>
       </c>
       <c r="E83" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="F83" t="s">
-        <v>157</v>
+        <v>129</v>
       </c>
       <c r="H83" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
@@ -3174,19 +3103,19 @@
         <v>1</v>
       </c>
       <c r="C84" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
       <c r="D84" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="E84" t="s">
-        <v>80</v>
+        <v>227</v>
       </c>
       <c r="F84" t="s">
-        <v>160</v>
+        <v>132</v>
       </c>
       <c r="H84" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
@@ -3197,19 +3126,19 @@
         <v>2</v>
       </c>
       <c r="C85" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
       <c r="D85" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="E85" t="s">
-        <v>161</v>
+        <v>227</v>
       </c>
       <c r="F85" t="s">
-        <v>162</v>
+        <v>133</v>
       </c>
       <c r="H85" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
@@ -3220,19 +3149,19 @@
         <v>3</v>
       </c>
       <c r="C86" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
       <c r="D86" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="E86" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F86" t="s">
-        <v>163</v>
+        <v>134</v>
       </c>
       <c r="H86" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
@@ -3243,19 +3172,19 @@
         <v>4</v>
       </c>
       <c r="C87" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
       <c r="D87" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="E87" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F87" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H87" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
@@ -3266,22 +3195,22 @@
         <v>1</v>
       </c>
       <c r="C88" t="s">
-        <v>164</v>
+        <v>135</v>
       </c>
       <c r="D88" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="E88" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F88" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="G88" t="s">
-        <v>167</v>
+        <v>138</v>
       </c>
       <c r="H88" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
@@ -3292,19 +3221,19 @@
         <v>1</v>
       </c>
       <c r="C89" t="s">
-        <v>164</v>
+        <v>135</v>
       </c>
       <c r="D89" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="E89" t="s">
-        <v>168</v>
+        <v>233</v>
       </c>
       <c r="F89" t="s">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="H89" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
@@ -3315,19 +3244,19 @@
         <v>1</v>
       </c>
       <c r="C90" t="s">
-        <v>164</v>
+        <v>135</v>
       </c>
       <c r="D90" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="E90" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F90" t="s">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="H90" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
@@ -3338,22 +3267,22 @@
         <v>1</v>
       </c>
       <c r="C91" t="s">
-        <v>171</v>
+        <v>141</v>
       </c>
       <c r="D91" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
       <c r="E91" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F91" t="s">
-        <v>173</v>
+        <v>143</v>
       </c>
       <c r="G91" t="s">
-        <v>174</v>
+        <v>144</v>
       </c>
       <c r="H91" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
@@ -3364,19 +3293,19 @@
         <v>2</v>
       </c>
       <c r="C92" t="s">
-        <v>171</v>
+        <v>141</v>
       </c>
       <c r="D92" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
       <c r="E92" t="s">
-        <v>12</v>
+        <v>226</v>
       </c>
       <c r="F92" t="s">
-        <v>175</v>
+        <v>145</v>
       </c>
       <c r="H92" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
@@ -3387,22 +3316,22 @@
         <v>1</v>
       </c>
       <c r="C93" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="D93" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="E93" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F93" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
       <c r="G93" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="H93" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
@@ -3413,19 +3342,19 @@
         <v>2</v>
       </c>
       <c r="C94" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="D94" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="E94" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F94" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="H94" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
@@ -3436,19 +3365,19 @@
         <v>3</v>
       </c>
       <c r="C95" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="D95" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="E95" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F95" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="H95" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.25">
@@ -3459,19 +3388,19 @@
         <v>4</v>
       </c>
       <c r="C96" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="D96" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="E96" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F96" t="s">
-        <v>182</v>
+        <v>152</v>
       </c>
       <c r="H96" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
@@ -3482,19 +3411,19 @@
         <v>5</v>
       </c>
       <c r="C97" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="D97" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="E97" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F97" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H97" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
@@ -3505,22 +3434,22 @@
         <v>1</v>
       </c>
       <c r="C98" t="s">
-        <v>183</v>
+        <v>153</v>
       </c>
       <c r="D98" t="s">
-        <v>184</v>
+        <v>154</v>
       </c>
       <c r="E98" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="F98" t="s">
-        <v>185</v>
+        <v>155</v>
       </c>
       <c r="G98" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
       <c r="H98" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
@@ -3531,19 +3460,19 @@
         <v>1</v>
       </c>
       <c r="C99" t="s">
-        <v>183</v>
+        <v>153</v>
       </c>
       <c r="D99" t="s">
-        <v>184</v>
+        <v>154</v>
       </c>
       <c r="E99" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F99" t="s">
-        <v>152</v>
+        <v>124</v>
       </c>
       <c r="H99" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.25">
@@ -3554,19 +3483,19 @@
         <v>1</v>
       </c>
       <c r="C100" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
       <c r="D100" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
       <c r="E100" t="s">
-        <v>189</v>
+        <v>109</v>
       </c>
       <c r="F100" t="s">
-        <v>190</v>
+        <v>159</v>
       </c>
       <c r="H100" t="s">
-        <v>259</v>
+        <v>224</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
@@ -3577,19 +3506,19 @@
         <v>1</v>
       </c>
       <c r="C101" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
       <c r="D101" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
       <c r="E101" t="s">
-        <v>191</v>
+        <v>109</v>
       </c>
       <c r="F101" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="H101" t="s">
-        <v>259</v>
+        <v>224</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.25">
@@ -3600,19 +3529,19 @@
         <v>1</v>
       </c>
       <c r="C102" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
       <c r="D102" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
       <c r="E102" t="s">
-        <v>193</v>
+        <v>109</v>
       </c>
       <c r="F102" t="s">
-        <v>194</v>
+        <v>161</v>
       </c>
       <c r="H102" t="s">
-        <v>259</v>
+        <v>224</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
@@ -3623,19 +3552,19 @@
         <v>1</v>
       </c>
       <c r="C103" t="s">
-        <v>195</v>
+        <v>162</v>
       </c>
       <c r="D103" t="s">
-        <v>196</v>
+        <v>163</v>
       </c>
       <c r="E103" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F103" t="s">
-        <v>197</v>
+        <v>164</v>
       </c>
       <c r="H103" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.25">
@@ -3646,19 +3575,19 @@
         <v>1</v>
       </c>
       <c r="C104" t="s">
-        <v>195</v>
+        <v>162</v>
       </c>
       <c r="D104" t="s">
-        <v>196</v>
+        <v>163</v>
       </c>
       <c r="E104" t="s">
-        <v>12</v>
+        <v>226</v>
       </c>
       <c r="F104" t="s">
-        <v>198</v>
+        <v>165</v>
       </c>
       <c r="H104" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.25">
@@ -3669,19 +3598,19 @@
         <v>1</v>
       </c>
       <c r="C105" t="s">
-        <v>195</v>
+        <v>162</v>
       </c>
       <c r="D105" t="s">
-        <v>196</v>
+        <v>163</v>
       </c>
       <c r="E105" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F105" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H105" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.25">
@@ -3692,19 +3621,19 @@
         <v>1</v>
       </c>
       <c r="C106" t="s">
-        <v>199</v>
+        <v>166</v>
       </c>
       <c r="D106" t="s">
-        <v>200</v>
+        <v>167</v>
       </c>
       <c r="E106" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F106" t="s">
-        <v>201</v>
+        <v>168</v>
       </c>
       <c r="H106" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.25">
@@ -3715,19 +3644,19 @@
         <v>2</v>
       </c>
       <c r="C107" t="s">
-        <v>199</v>
+        <v>166</v>
       </c>
       <c r="D107" t="s">
-        <v>200</v>
+        <v>167</v>
       </c>
       <c r="E107" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F107" t="s">
-        <v>202</v>
+        <v>169</v>
       </c>
       <c r="H107" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.25">
@@ -3738,22 +3667,22 @@
         <v>1</v>
       </c>
       <c r="C108" t="s">
-        <v>203</v>
+        <v>170</v>
       </c>
       <c r="D108" t="s">
-        <v>204</v>
+        <v>171</v>
       </c>
       <c r="E108" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F108" t="s">
-        <v>205</v>
+        <v>172</v>
       </c>
       <c r="G108" t="s">
-        <v>206</v>
+        <v>173</v>
       </c>
       <c r="H108" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.25">
@@ -3764,19 +3693,19 @@
         <v>1</v>
       </c>
       <c r="C109" t="s">
-        <v>203</v>
+        <v>170</v>
       </c>
       <c r="D109" t="s">
-        <v>204</v>
+        <v>171</v>
       </c>
       <c r="E109" t="s">
-        <v>72</v>
+        <v>232</v>
       </c>
       <c r="F109" t="s">
-        <v>207</v>
+        <v>174</v>
       </c>
       <c r="H109" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
@@ -3787,19 +3716,19 @@
         <v>1</v>
       </c>
       <c r="C110" t="s">
-        <v>203</v>
+        <v>170</v>
       </c>
       <c r="D110" t="s">
-        <v>204</v>
+        <v>171</v>
       </c>
       <c r="E110" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="F110" t="s">
-        <v>208</v>
+        <v>175</v>
       </c>
       <c r="H110" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
@@ -3810,19 +3739,19 @@
         <v>1</v>
       </c>
       <c r="C111" t="s">
-        <v>203</v>
+        <v>170</v>
       </c>
       <c r="D111" t="s">
-        <v>204</v>
+        <v>171</v>
       </c>
       <c r="E111" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F111" t="s">
-        <v>209</v>
+        <v>176</v>
       </c>
       <c r="H111" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
@@ -3833,19 +3762,19 @@
         <v>1</v>
       </c>
       <c r="C112" t="s">
-        <v>210</v>
+        <v>177</v>
       </c>
       <c r="D112" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="E112" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F112" t="s">
-        <v>212</v>
+        <v>179</v>
       </c>
       <c r="H112" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.25">
@@ -3856,19 +3785,19 @@
         <v>1</v>
       </c>
       <c r="C113" t="s">
-        <v>210</v>
+        <v>177</v>
       </c>
       <c r="D113" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="E113" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F113" t="s">
-        <v>213</v>
+        <v>180</v>
       </c>
       <c r="H113" t="s">
-        <v>257</v>
+        <v>222</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.25">
@@ -3879,19 +3808,19 @@
         <v>1</v>
       </c>
       <c r="C114" t="s">
-        <v>214</v>
+        <v>181</v>
       </c>
       <c r="D114" t="s">
-        <v>215</v>
+        <v>182</v>
       </c>
       <c r="E114" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F114" t="s">
-        <v>216</v>
+        <v>183</v>
       </c>
       <c r="H114" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.25">
@@ -3902,19 +3831,19 @@
         <v>2</v>
       </c>
       <c r="C115" t="s">
-        <v>214</v>
+        <v>181</v>
       </c>
       <c r="D115" t="s">
-        <v>215</v>
+        <v>182</v>
       </c>
       <c r="E115" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F115" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H115" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.25">
@@ -3925,19 +3854,19 @@
         <v>1</v>
       </c>
       <c r="C116" t="s">
-        <v>217</v>
+        <v>184</v>
       </c>
       <c r="D116" t="s">
-        <v>218</v>
+        <v>185</v>
       </c>
       <c r="E116" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="F116" t="s">
-        <v>219</v>
+        <v>186</v>
       </c>
       <c r="H116" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.25">
@@ -3948,19 +3877,19 @@
         <v>2</v>
       </c>
       <c r="C117" t="s">
-        <v>217</v>
+        <v>184</v>
       </c>
       <c r="D117" t="s">
-        <v>218</v>
+        <v>185</v>
       </c>
       <c r="E117" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="F117" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H117" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.25">
@@ -3971,22 +3900,22 @@
         <v>1</v>
       </c>
       <c r="C118" t="s">
-        <v>221</v>
+        <v>187</v>
       </c>
       <c r="D118" t="s">
-        <v>222</v>
+        <v>188</v>
       </c>
       <c r="E118" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F118" t="s">
-        <v>223</v>
+        <v>189</v>
       </c>
       <c r="G118" t="s">
-        <v>224</v>
+        <v>190</v>
       </c>
       <c r="H118" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.25">
@@ -3997,19 +3926,19 @@
         <v>2</v>
       </c>
       <c r="C119" t="s">
-        <v>221</v>
+        <v>187</v>
       </c>
       <c r="D119" t="s">
-        <v>222</v>
+        <v>188</v>
       </c>
       <c r="E119" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F119" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H119" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.25">
@@ -4020,19 +3949,19 @@
         <v>1</v>
       </c>
       <c r="C120" t="s">
-        <v>225</v>
+        <v>191</v>
       </c>
       <c r="D120" t="s">
-        <v>226</v>
+        <v>192</v>
       </c>
       <c r="E120" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
       <c r="F120" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="H120" t="s">
-        <v>259</v>
+        <v>224</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.25">
@@ -4043,22 +3972,23 @@
         <v>2</v>
       </c>
       <c r="C121" t="s">
-        <v>225</v>
+        <v>191</v>
       </c>
       <c r="D121" t="s">
-        <v>226</v>
+        <v>192</v>
       </c>
       <c r="E121" t="s">
-        <v>21</v>
+        <v>230</v>
       </c>
       <c r="F121" t="s">
-        <v>227</v>
+        <v>193</v>
       </c>
       <c r="H121" t="s">
-        <v>259</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="E1:E121" xr:uid="{FC2EDDBB-A715-1D44-9E74-98BE5ED7B607}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H72 H75:H121" xr:uid="{43A2730F-810B-D042-B533-EDFBEA84A167}">

</xml_diff>